<commit_message>
feat: CRM fixes + asset spreadsheet update + config
</commit_message>
<xml_diff>
--- a/docs/Device_Inventory.xlsx
+++ b/docs/Device_Inventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10503"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fangkaryuan/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fangkaryuan/cwc2.0/citadel-cwc-portal/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CBF4B858-32E8-8D4F-B472-AF5B906360A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24EE8A7C-379E-B342-8148-08B3CC2FBDFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="800" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Laptops | Desktops" sheetId="1" r:id="rId1"/>
@@ -1266,7 +1266,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1294,6 +1294,17 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri (Body)"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1373,7 +1384,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1414,8 +1425,15 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1696,7 +1714,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:XES53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1882,7 +1899,7 @@
       <c r="R3" s="4"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="20" t="s">
         <v>41</v>
       </c>
       <c r="B4" s="4" t="s">
@@ -2303,55 +2320,55 @@
       </c>
       <c r="R11" s="4"/>
     </row>
-    <row r="12" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4" t="s">
+    <row r="12" spans="1:18" s="24" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="23"/>
+      <c r="B12" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="23" t="s">
         <v>106</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="I12" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4" t="b">
+      <c r="J12" s="23"/>
+      <c r="K12" s="23" t="b">
         <v>0</v>
       </c>
-      <c r="L12" s="4" t="s">
+      <c r="L12" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="M12" s="4" t="s">
+      <c r="M12" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="N12" s="4" t="s">
+      <c r="N12" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="O12" s="4" t="s">
+      <c r="O12" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="P12" s="4" t="s">
+      <c r="P12" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="Q12" s="4" t="s">
+      <c r="Q12" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="R12" s="4" t="s">
+      <c r="R12" s="23" t="s">
         <v>109</v>
       </c>
     </row>
@@ -2719,101 +2736,101 @@
       </c>
       <c r="R19" s="4"/>
     </row>
-    <row r="20" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="20" t="s">
+    <row r="20" spans="1:18" s="22" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="21" t="s">
         <v>159</v>
       </c>
-      <c r="D20" s="20" t="s">
+      <c r="D20" s="21" t="s">
         <v>160</v>
       </c>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20" t="s">
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="H20" s="20" t="s">
+      <c r="H20" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="I20" s="20" t="s">
+      <c r="I20" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="J20" s="20"/>
-      <c r="K20" s="20" t="b">
+      <c r="J20" s="21"/>
+      <c r="K20" s="21" t="b">
         <v>1</v>
       </c>
-      <c r="L20" s="20" t="s">
+      <c r="L20" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="M20" s="20" t="s">
+      <c r="M20" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="N20" s="20" t="s">
+      <c r="N20" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="O20" s="20" t="s">
+      <c r="O20" s="21" t="s">
         <v>161</v>
       </c>
-      <c r="P20" s="20" t="s">
+      <c r="P20" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="Q20" s="20" t="s">
+      <c r="Q20" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="R20" s="20"/>
+      <c r="R20" s="21"/>
     </row>
-    <row r="21" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="20" t="s">
+    <row r="21" spans="1:18" s="22" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="21" t="s">
         <v>163</v>
       </c>
-      <c r="B21" s="20" t="s">
+      <c r="B21" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="C21" s="20" t="s">
+      <c r="C21" s="21" t="s">
         <v>159</v>
       </c>
-      <c r="D21" s="20" t="s">
+      <c r="D21" s="21" t="s">
         <v>160</v>
       </c>
-      <c r="E21" s="20"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20" t="s">
+      <c r="E21" s="21"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="H21" s="20" t="s">
+      <c r="H21" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="I21" s="20" t="s">
+      <c r="I21" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="J21" s="20"/>
-      <c r="K21" s="20" t="b">
+      <c r="J21" s="21"/>
+      <c r="K21" s="21" t="b">
         <v>1</v>
       </c>
-      <c r="L21" s="20" t="s">
+      <c r="L21" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="M21" s="20" t="s">
+      <c r="M21" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="N21" s="20" t="s">
+      <c r="N21" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="O21" s="20" t="s">
+      <c r="O21" s="21" t="s">
         <v>161</v>
       </c>
-      <c r="P21" s="20" t="s">
+      <c r="P21" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="Q21" s="20" t="s">
+      <c r="Q21" s="21" t="s">
         <v>165</v>
       </c>
-      <c r="R21" s="20"/>
+      <c r="R21" s="21"/>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
@@ -2869,97 +2886,97 @@
       </c>
       <c r="R22" s="10"/>
     </row>
-    <row r="23" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="4"/>
-      <c r="B23" s="4" t="s">
+    <row r="23" spans="1:18" s="24" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="23"/>
+      <c r="B23" s="23" t="s">
         <v>158</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="23" t="s">
         <v>159</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="23" t="s">
         <v>160</v>
       </c>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4" t="s">
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="H23" s="4" t="s">
+      <c r="H23" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="I23" s="4" t="s">
+      <c r="I23" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4" t="b">
+      <c r="J23" s="23"/>
+      <c r="K23" s="23" t="b">
         <v>1</v>
       </c>
-      <c r="L23" s="4" t="s">
+      <c r="L23" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="M23" s="4" t="s">
+      <c r="M23" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="N23" s="4" t="s">
+      <c r="N23" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="O23" s="4" t="s">
+      <c r="O23" s="23" t="s">
         <v>161</v>
       </c>
-      <c r="P23" s="4" t="s">
+      <c r="P23" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="Q23" s="4" t="s">
+      <c r="Q23" s="23" t="s">
         <v>162</v>
       </c>
-      <c r="R23" s="4"/>
+      <c r="R23" s="23"/>
     </row>
-    <row r="24" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4" t="s">
+    <row r="24" spans="1:18" s="24" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="23"/>
+      <c r="B24" s="23" t="s">
         <v>164</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="23" t="s">
         <v>159</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="23" t="s">
         <v>160</v>
       </c>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4" t="s">
+      <c r="E24" s="23"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="H24" s="4" t="s">
+      <c r="H24" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="I24" s="4" t="s">
+      <c r="I24" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4" t="b">
+      <c r="J24" s="23"/>
+      <c r="K24" s="23" t="b">
         <v>1</v>
       </c>
-      <c r="L24" s="4" t="s">
+      <c r="L24" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="M24" s="4" t="s">
+      <c r="M24" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="N24" s="4" t="s">
+      <c r="N24" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="O24" s="4" t="s">
+      <c r="O24" s="23" t="s">
         <v>161</v>
       </c>
-      <c r="P24" s="4" t="s">
+      <c r="P24" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="Q24" s="4" t="s">
+      <c r="Q24" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="R24" s="4"/>
+      <c r="R24" s="23"/>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
@@ -3169,7 +3186,7 @@
       </c>
       <c r="R28" s="5"/>
     </row>
-    <row r="29" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
         <v>204</v>
       </c>
@@ -3381,7 +3398,7 @@
       </c>
       <c r="R32" s="5"/>
     </row>
-    <row r="33" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
         <v>232</v>
       </c>
@@ -3435,111 +3452,111 @@
       </c>
       <c r="R33" s="5"/>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A34" s="5" t="s">
+    <row r="34" spans="1:18" s="24" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="25" t="s">
         <v>238</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="25" t="s">
         <v>239</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D34" s="25" t="s">
         <v>132</v>
       </c>
-      <c r="E34" s="14" t="s">
+      <c r="E34" s="26" t="s">
         <v>240</v>
       </c>
-      <c r="F34" s="14" t="s">
+      <c r="F34" s="26" t="s">
         <v>241</v>
       </c>
-      <c r="G34" s="14" t="s">
+      <c r="G34" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="H34" s="5" t="s">
+      <c r="H34" s="25" t="s">
         <v>242</v>
       </c>
-      <c r="I34" s="5" t="s">
+      <c r="I34" s="25" t="s">
         <v>243</v>
       </c>
-      <c r="J34" s="5"/>
-      <c r="K34" s="5" t="b">
+      <c r="J34" s="25"/>
+      <c r="K34" s="25" t="b">
         <v>1</v>
       </c>
-      <c r="L34" s="5" t="s">
+      <c r="L34" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="M34" s="5" t="s">
+      <c r="M34" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="N34" s="5" t="s">
+      <c r="N34" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="O34" s="5" t="s">
+      <c r="O34" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="P34" s="5" t="s">
+      <c r="P34" s="25" t="s">
         <v>180</v>
       </c>
-      <c r="Q34" s="5" t="s">
+      <c r="Q34" s="25" t="s">
         <v>244</v>
       </c>
-      <c r="R34" s="5"/>
+      <c r="R34" s="25"/>
     </row>
-    <row r="35" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="5" t="s">
+    <row r="35" spans="1:18" s="24" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="25" t="s">
         <v>245</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="25" t="s">
         <v>239</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C35" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="D35" s="25" t="s">
         <v>132</v>
       </c>
-      <c r="E35" s="5" t="s">
+      <c r="E35" s="25" t="s">
         <v>240</v>
       </c>
-      <c r="F35" s="5" t="s">
+      <c r="F35" s="25" t="s">
         <v>241</v>
       </c>
-      <c r="G35" s="5" t="s">
+      <c r="G35" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="H35" s="5" t="s">
+      <c r="H35" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="I35" s="5" t="s">
+      <c r="I35" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="J35" s="5" t="s">
+      <c r="J35" s="25" t="s">
         <v>246</v>
       </c>
-      <c r="K35" s="5" t="b">
+      <c r="K35" s="25" t="b">
         <v>1</v>
       </c>
-      <c r="L35" s="5" t="s">
+      <c r="L35" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="M35" s="5" t="s">
+      <c r="M35" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="N35" s="5" t="s">
+      <c r="N35" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="O35" s="5" t="s">
+      <c r="O35" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="P35" s="5" t="s">
+      <c r="P35" s="25" t="s">
         <v>180</v>
       </c>
-      <c r="Q35" s="5" t="s">
+      <c r="Q35" s="25" t="s">
         <v>244</v>
       </c>
-      <c r="R35" s="5" t="s">
+      <c r="R35" s="25" t="s">
         <v>247</v>
       </c>
     </row>
@@ -3697,7 +3714,7 @@
       </c>
       <c r="R38" s="8"/>
     </row>
-    <row r="39" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A39" s="9" t="s">
         <v>276</v>
       </c>
@@ -3751,7 +3768,7 @@
       </c>
       <c r="R39" s="2"/>
     </row>
-    <row r="40" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
         <v>284</v>
       </c>
@@ -4065,7 +4082,7 @@
       </c>
       <c r="R45" s="7"/>
     </row>
-    <row r="46" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A46" s="7" t="s">
         <v>328</v>
       </c>
@@ -4119,7 +4136,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="47" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
         <v>335</v>
       </c>
@@ -4383,7 +4400,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="52" spans="1:16373" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:16373" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
         <v>373</v>
       </c>
@@ -20848,44 +20865,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:R53" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="7">
-      <filters>
-        <filter val="adly.mohamed@citadelgroup.com.my"/>
-        <filter val="ahmad.zuhayri@citadelgroup.com.my"/>
-        <filter val="alain.boey@citadelgroup.com.my"/>
-        <filter val="alan.ling@citadelgroup.com.my"/>
-        <filter val="cheehao.wong@citadelgroup.com.my"/>
-        <filter val="emily.chow@citadelgroup.com.my"/>
-        <filter val="fadhli.amran@citadelgroup.com.my"/>
-        <filter val="fangkhai.foo@citadelgroup.com.my"/>
-        <filter val="girling.liong@citadelgroup.com.my"/>
-        <filter val="irina.kamarzan@citadelgroup.com.my"/>
-        <filter val="j.medina@citadelgroup.com.my"/>
-        <filter val="joyce.loh@citadelgroup.com.my"/>
-        <filter val="juliana.jalil@citadelgroup.com.my"/>
-        <filter val="kamilah.hanif@citadelgroup.com.my"/>
-        <filter val="karyuan.fang@citadelgroup.com.my"/>
-        <filter val="khaliesah.badruddin@citadelgroup.com.my"/>
-        <filter val="michelle.weng@citadelgroup.com.my"/>
-        <filter val="mingkai.tham@citadelgroup.com.my"/>
-        <filter val="natalya.erika@citadelgroup.com.my"/>
-        <filter val="natasha.dealwis@citadelgroup.com.my"/>
-        <filter val="naveen.ahmad@citadelgroup.com.my"/>
-        <filter val="nick.tan@citadelgroup.com.my"/>
-        <filter val="nurnafisah.sharudin@citadelgroup.com.my"/>
-        <filter val="rajna.anthony@citadelgroup.com.my"/>
-        <filter val="raymond.kueh@citadelgroup.com.my"/>
-        <filter val="rohani.munir@citadelgroup.com.my"/>
-        <filter val="saravanan.ramaiah@citadelgroup.com.my"/>
-        <filter val="sasha.nair@citadelgroup.com.my"/>
-        <filter val="Server Admin"/>
-        <filter val="shah.musa@citadelgroup.com.my"/>
-        <filter val="shamsuria.shamsuri@citadelgroup.com.my"/>
-        <filter val="soraya.rozali@citadelgroup.com.my"/>
-        <filter val="zac.ashari@citadelgroup.com.my"/>
-        <filter val="zahidah.rashid@citadelgroup.com.my"/>
-      </filters>
-    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R53">
       <sortCondition ref="P1:P53"/>
     </sortState>

</xml_diff>